<commit_message>
docs(conversacion-6): cruce con las notas a mano + Excel de preguntas al dia
Las 3 imagenes son las notas que Jorge tomo durante la misma reunion. Sirven
de contraste independiente contra lo que se saco de los audios y el cruce da
1:1: los 15 apuntes caen todos dentro de A1-01..A1-20.

Un solo item nuevo — el segundo pito. Son DOS, no uno: uno cuando el paquete
tiene pre-alerta y otro cuando el tracking ya existia. Incorporado a A1-10.

Las dos tachaduras de las notas apuntan al mismo bug: "Tab" tachado y
reemplazado por "enter", y "Grabar" tachado y reemplazado por "seleccionar".
De los 15 apuntes, cinco son A1-01 o su consecuencia directa.

Excel de preguntas actualizado: salen las tres que Yusef contesto en la
reunion (cambio de servicio, moneda de los cargos, redondeo) y entran 14
nuevas de los dos audios. Quedan 23: 4 altas, 18 medias, 1 baja.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FJgcheJN9spiFwv9KGNUZS
</commit_message>
<xml_diff>
--- a/docs/entregables/preguntas_para_yusef.xlsx
+++ b/docs/entregables/preguntas_para_yusef.xlsx
@@ -439,7 +439,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="4" min="1" max="1" bestFit="1" customWidth="1"/>
@@ -453,7 +453,7 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>Preguntas para Yusef — 06 de Agosto de 2026</t>
+          <t>Preguntas para Yusef — 08 de Agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -471,72 +471,49 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
-    <row customHeight="1" ht="78" r="5">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>En la reunión del 8 de agosto ya contestaste tres: el cambio de servicio (L.100), la moneda de los cargos y el redondeo de libras. Esas ya no están acá.</t>
+        </is>
+      </c>
+    </row>
+    <row customHeight="1" ht="78" r="5"/>
+    <row customHeight="1" ht="78" r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Urgencia</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Tema</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Pregunta</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Lo que sabemos hoy</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>TU RESPUESTA</t>
-        </is>
-      </c>
-    </row>
-    <row customHeight="1" ht="78" r="6">
-      <c r="A6" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Cambio de servicio</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>En tu hoja el cambio de servicio dice 5 y el titulo dice L100, con la nota "pasarlo a dolares". En el sistema esta cargado en $15. ¿Cual queda?</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>Este cargo se genera SOLO, en una nota de debito, cada vez que se factura un paquete al que le cambiaron el servicio. Mientras no nos digas, sigue cobrando los $15 — que es el triple de los 5 de tu hoja.</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
     </row>
     <row customHeight="1" ht="78" r="7">
       <c r="A7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
@@ -545,17 +522,17 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Moneda de 10 cargos</t>
+          <t>Formato del N° de recepcion</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Necesitamos la moneda de 10 cargos de tu hoja. Estan en la HOJA 4 con la duda de cada uno y una columna para que escribas $ o LPS.</t>
+          <t>Dijiste que al numero de recepcion le falta el MES, y que ya nos lo habias mandado. ¿Nos pasas el formato exacto? Ejemplo de como quedaria un paquete recibido en Miami en agosto 2026.</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>En tu hoja pusiste la leyenda "precios en $" y "precios en lempiras" pero las celdas de precio quedaron sin colorear, asi que un 5 no dice si son 5 dolares o 5 lempiras. Ya cargamos los 5 que si dejaste claros con una nota escrita.</t>
+          <t>Hoy el numero es RM + anio + correlativo de 6 digitos: RM0002026000010. El correlativo reinicia cada enero. Cambiar el formato toca todos los numeros ya generados, por eso no lo inventamos nosotros.</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -566,7 +543,7 @@
     </row>
     <row customHeight="1" ht="78" r="8">
       <c r="A8" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
@@ -575,17 +552,17 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Recolecta: ¿zona o plano?</t>
+          <t>Redondeo de libras</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Vos pediste que la recolecta se cobrara POR ZONA en vez de $35 fijos, y asi esta hecho. Pero tu hoja nueva dice 35 plano. ¿Cual mandamos?</t>
+          <t>La regla que diste (1.09 se cobra 1.0, 1.10 se cobra 1.5, 1.60 se cobra 2.0) es para escalones de MEDIA libra. Si armas una tarifa con escalon de 1 libra entera, ¿la tolerancia sigue siendo 0.09?</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Hoy el sistema tiene una tabla de tarifas de recolecta por zona/distancia, que es lo que pediste en su momento. Si mandamos el 35 plano, esa tabla deja de usarse.</t>
+          <t>Hoy el sistema no redondea: cobra el peso exacto. Cuando actives el escalonado va a redondear, y necesitamos la regla completa para no cobrarte de mas a vos ni de menos al cliente.</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
@@ -596,26 +573,26 @@
     </row>
     <row customHeight="1" ht="78" r="9">
       <c r="A9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Revisar los precios cargados</t>
+          <t>Recolecta: ¿zona o plano?</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>En la HOJA 2 esta TODO lo que quedo cargado de tu tabla, leido directo del sistema. Es literalmente lo que va a cobrar. ¿Esta bien?</t>
+          <t>Vos pediste que la recolecta se cobrara POR ZONA en vez de $35 fijos, y asi esta hecho. En el audio dijiste "$35 normal, pero hay clientes con descuento". ¿La recolecta de MIAMI y la de HONDURAS son dos cosas distintas?</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>Tomamos la hoja PROPUESTA de "precios por categoria 2026.xlsx". Si algo esta mal, escribilo en la ultima columna de esa hoja.</t>
+          <t>Hoy el sistema tiene una tabla de tarifas de recolecta por zona/distancia, que es lo que pediste en su momento. Si el $35 de Miami es otro cargo aparte, conviven los dos sin problema.</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -626,26 +603,26 @@
     </row>
     <row customHeight="1" ht="78" r="10">
       <c r="A10" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Las categorías no bajan de escalón</t>
+          <t>Manejo y gastos de destino</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Un cliente "Clientes Amigos" con 200 libras de CER paga $4.20 la libra ($840) mientras el publico paga $3.50 ($700). ¿Es asi, o las categorias tambien deberian bajar de escalon?</t>
+          <t>Tu hoja dice textual "ponerlo lps1 mas isv", pero en el audio dijiste que es "parecido al de ajuste", y ajuste es en dolares. ¿Lempiras o dolares?</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Tu tabla da un solo precio por categoria (columna NORMAL) y los tarifarios escalonados los declaraste solo para el Precio Normal. Lo cargamos literal a como lo mandaste, pero el resultado es que un amigo paga mas que un cliente de mostrador en paquetes grandes.</t>
+          <t>Lo dejamos en Lempiras, que es lo que dice la nota escrita de tu hoja. Es el unico cargo donde el audio y la hoja no coinciden.</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
@@ -656,7 +633,7 @@
     </row>
     <row customHeight="1" ht="78" r="11">
       <c r="A11" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
@@ -665,17 +642,17 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>CKM cae en dos reglas</t>
+          <t>Retornado de Miami</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Para CKM, ¿cual minimo manda: los L.200, el de libras, o el que resulte MAYOR de los dos?</t>
+          <t>Dijiste "$5 es como un precio minimo" y que si va por USPS sube a $15 porque hay que pagar motorista. ¿Son dos cargos distintos, o uno con minimo de $5?</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>En el audio dijiste "los servicios serie CK son 200 lempiras ya con ISV" (aplica a CKA y CKM) y tambien "el maritimo lo tenemos estipulado en cantidad de libras" (aplica a CEM y CKM). CKM es las dos cosas. En tu tabla le pusiste L.173.91, asi que cargamos ese.</t>
+          <t>Cargado a $5. Si son dos, los damos de alta por separado y en Miami eligen cual aplica.</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -686,7 +663,7 @@
     </row>
     <row customHeight="1" ht="78" r="12">
       <c r="A12" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
@@ -695,17 +672,17 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Mínimo en libras de CEM y CKM</t>
+          <t>Entrada y salida (IN &amp; OUT)</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>¿Hace falta todavia un minimo en LIBRAS para CEM y CKM, o con el minimo en dinero de tu tabla ya esta?</t>
+          <t>Dijiste que es "de 10 a 5 depende". ¿De que depende — del tamano del paquete, del cliente, de la cantidad?</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>Tu tabla trae el minimo en dinero (L.200 con ISV) pero no el de libras. En la practica el escalonado ya cubre el paquete chico: un CEM de 2 libras paga $4.50 la libra. Documentado en abril: CEM = 8 libras, CKM = 20 libras. En el audio dijiste 3 o 4 libras.</t>
+          <t>Es cuando el cliente recibe en Miami y lo recoge el mismo. Nos diste el ejemplo de 3 paquetes a $5 cada uno.</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
@@ -716,7 +693,7 @@
     </row>
     <row customHeight="1" ht="78" r="13">
       <c r="A13" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
@@ -725,17 +702,17 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Regular y VIP</t>
+          <t>Flete Mexico y etiqueta internacional</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Hay 8 clientes en las categorias "Regular" y "VIP", que no aparecen en tu tabla. ¿A cual de las nuevas los pasamos, o los dejamos como estan?</t>
+          <t>Dos cosas: (a) el flete de Mexico a Honduras, ¿en que moneda? (b) la creacion de etiqueta internacional que mencionaste, ¿que precio y en que moneda?</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Por ahora se quedaron con los precios viejos, que son mas bajos que los de lista. Las categorias de tu tabla son: Clientes Amigos, doTERRA/Farmasi, Familia, Mayoristas, Personal de CEC, Shein, Revendedores y Sin Cobro Minimo.</t>
+          <t>El flete Mexico esta en tu hoja con precio pero sin moneda. La etiqueta internacional no esta ni en la hoja ni en el sistema — la mencionaste como parte de los retornados de Miami.</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -746,7 +723,7 @@
     </row>
     <row customHeight="1" ht="78" r="14">
       <c r="A14" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
@@ -755,17 +732,17 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Mayoristas incompleto</t>
+          <t>Buscar cliente por los ultimos digitos</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>De MAYORISTAS solo vino el precio de CKM ($1.50). Los otros cuatro servicios vinieron en cero. ¿Que cobran los mayoristas en CER, CKA, EXPRESS y CEM?</t>
+          <t>Pediste que se pueda escribir solo el final del codigo (2867, o hasta un solo 6) y que caiga. Con codigos de 5 digitos, escribir un 6 va a traer cientos. ¿Mostramos todos los que terminan en 6, o priorizamos el que coincide exacto?</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>Mientras tanto esos cuatro siguen con los valores viejos del sistema, que no salieron de tu tabla. FAMILIA y REVENDEDORES vinieron todos en cero, asi que sus clientes pagan precio de lista.</t>
+          <t>Asi trabajan hoy en el sistema viejo, y los codigos viejos de 4 digitos no se van a migrar.</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
@@ -776,7 +753,7 @@
     </row>
     <row customHeight="1" ht="78" r="15">
       <c r="A15" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
@@ -785,17 +762,17 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>PINs de los supervisores</t>
+          <t>Guardar: ¿F8 o F10?</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>El codigo del supervisor ya esta funcionando. ¿A quienes les asignamos PIN? Pueden tenerlo: Administrador, Supervisor Caja, Supervisor Pre-Factura y Supervisor de Servicio al Cliente.</t>
+          <t>En etiquetar guardar es F8, pero en pre-facturas, ventas, caja y financiamientos es F10 — y vos apretaste F10 sin pensarlo. ¿Lo pasamos todo a F10?</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>Un administrador se los asigna desde la pantalla de usuarios y despues cada supervisor lo cambia por uno que solo el sepa. Mientras no lo cambie, el administrador conoce el PIN con el que ese supervisor autoriza — la pantalla de usuarios marca a quienes les falta cambiarlo.</t>
+          <t>F8 en el resto del sistema es "exportar a Excel". Si cambiamos, hay que avisarle a Miami que ya tiene el F8 en el dedo.</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -806,7 +783,7 @@
     </row>
     <row customHeight="1" ht="78" r="16">
       <c r="A16" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
@@ -815,17 +792,17 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Probar la etiqueta impresa</t>
+          <t>Peso por caja</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Imprimi una etiqueta y decinos dos cosas: (1) si no se corta nada, sobre todo en un paquete que traiga tercero Y driver, que es el que mas campos lleva; (2) si el lector escanea bien el codigo de barras.</t>
+          <t>Si son 2 cajas, ¿preferis que salgan las 2 lineas de peso y medidas de una vez, o un boton "agregar" que las va sumando de a una?</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Los 11 campos van con la jerarquia de tamanos que marcaste. El codigo de barras quedo en 0.20 pulgadas de alto, que es el minimo practico para lectores de mano — es lo unico que no podemos probar nosotros. Los campos estan en la hoja 3.</t>
+          <t>Hoy pide una sola linea aunque sean varias cajas. Vos mencionaste las dos formas y dejaste elegir.</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
@@ -836,29 +813,389 @@
     </row>
     <row customHeight="1" ht="78" r="17">
       <c r="A17" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Bajar la cantidad de cajas</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Si un paquete tiene 5 cajas y alguien lo baja a 2, las otras 3 se borran. ¿Que hacemos si alguna de esas ya esta facturada o entregada?</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Hoy no se borra ninguna y quedan registros de mas, que es el error que viste. Lo mas seguro es no dejar borrar una caja ya facturada y avisar por que.</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row customHeight="1" ht="78" r="18">
+      <c r="A18" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Origen del paquete</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>El campo de origen (Estados Unidos / China) esta en pantalla sin definir. ¿Que origenes van, y cambia algo del cobro segun el origen?</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Dijiste "como ahorita estamos en Estados Unidos, pero ya va a abrir China".</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row customHeight="1" ht="78" r="19">
+      <c r="A19" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Listas que quedaste de mandar</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Nos faltan tres listas tuyas: (a) motivos de retencion completos — sabemos que falta "solicitado por el cliente para retorno"; (b) las notas predeterminadas de pre-factura, caja y servicio al cliente; (c) las grabaciones de voz para la alerta de pre-alerta.</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Los motivos y las notas van a quedar editables por vos, asi que podes agregarlos vos mismo despues. Las grabaciones son las que hizo tu senora en 2022 — dijiste que las volvias a grabar.</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row customHeight="1" ht="78" r="20">
+      <c r="A20" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Sonidos de etiquetar</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Te vamos a pasar una lista de sonidos para que elijas el de ERROR (el "feo", para cuando el paquete no es del tipo de envio de la sesion). ¿Preferis elegir vos o te proponemos uno?</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>El pin agradable que ya suena lo aprobaste. Faltan: el pito de "este tracking ya existia", el de error, y el pin antes de que salga cada modal.</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row customHeight="1" ht="78" r="21">
+      <c r="A21" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Revisar los precios cargados</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>En la HOJA 2 esta TODO lo que quedo cargado de tu tabla, leido directo del sistema. Es literalmente lo que va a cobrar. ¿Esta bien?</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Tomamos la hoja PROPUESTA de "precios por categoria 2026.xlsx". Si algo esta mal, escribilo en la ultima columna de esa hoja.</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row customHeight="1" ht="78" r="22">
+      <c r="A22" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Las categorías no bajan de escalón</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Un cliente "Clientes Amigos" con 200 libras de CER paga $4.20 la libra ($840) mientras el publico paga $3.50 ($700). ¿Es asi, o las categorias tambien deberian bajar de escalon?</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Tu tabla da un solo precio por categoria (columna NORMAL) y los tarifarios escalonados los declaraste solo para el Precio Normal. Lo cargamos literal a como lo mandaste, pero el resultado es que un amigo paga mas que un cliente de mostrador en paquetes grandes.</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row customHeight="1" ht="78" r="23">
+      <c r="A23" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>CKM cae en dos reglas</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Para CKM, ¿cual minimo manda: los L.200, el de libras, o el que resulte MAYOR de los dos?</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>En el audio dijiste "los servicios serie CK son 200 lempiras ya con ISV" (aplica a CKA y CKM) y tambien "el maritimo lo tenemos estipulado en cantidad de libras" (aplica a CEM y CKM). CKM es las dos cosas. En tu tabla le pusiste L.173.91, asi que cargamos ese.</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row customHeight="1" ht="78" r="24">
+      <c r="A24" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Mínimo en libras de CEM y CKM</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>¿Hace falta todavia un minimo en LIBRAS para CEM y CKM, o con el minimo en dinero de tu tabla ya esta?</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Tu tabla trae el minimo en dinero (L.200 con ISV) pero no el de libras. En la practica el escalonado ya cubre el paquete chico: un CEM de 2 libras paga $4.50 la libra. Documentado en abril: CEM = 8 libras, CKM = 20 libras. En el audio dijiste 3 o 4 libras.</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row customHeight="1" ht="78" r="25">
+      <c r="A25" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Regular y VIP</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Hay 8 clientes en las categorias "Regular" y "VIP", que no aparecen en tu tabla. ¿A cual de las nuevas los pasamos, o los dejamos como estan?</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>Por ahora se quedaron con los precios viejos, que son mas bajos que los de lista. Las categorias de tu tabla son: Clientes Amigos, doTERRA/Farmasi, Familia, Mayoristas, Personal de CEC, Shein, Revendedores y Sin Cobro Minimo.</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row customHeight="1" ht="78" r="26">
+      <c r="A26" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Mayoristas incompleto</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>De MAYORISTAS solo vino el precio de CKM ($1.50). Los otros cuatro servicios vinieron en cero. ¿Que cobran los mayoristas en CER, CKA, EXPRESS y CEM?</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>Mientras tanto esos cuatro siguen con los valores viejos del sistema, que no salieron de tu tabla. FAMILIA y REVENDEDORES vinieron todos en cero, asi que sus clientes pagan precio de lista.</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row customHeight="1" ht="78" r="27">
+      <c r="A27" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>PINs de los supervisores</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>El codigo del supervisor ya esta funcionando. ¿A quienes les asignamos PIN? Pueden tenerlo: Administrador, Supervisor Caja, Supervisor Pre-Factura y Supervisor de Servicio al Cliente.</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Un administrador se los asigna desde la pantalla de usuarios y despues cada supervisor lo cambia por uno que solo el sepa. Mientras no lo cambie, el administrador conoce el PIN con el que ese supervisor autoriza — la pantalla de usuarios marca a quienes les falta cambiarlo.</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row customHeight="1" ht="78" r="28">
+      <c r="A28" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Probar la etiqueta impresa</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Imprimi una etiqueta y decinos dos cosas: (1) si no se corta nada, sobre todo en un paquete que traiga tercero Y driver, que es el que mas campos lleva; (2) si el lector escanea bien el codigo de barras.</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Los 11 campos van con la jerarquia de tamanos que marcaste. El codigo de barras quedo en 0.20 pulgadas de alto, que es el minimo practico para lectores de mano — es lo unico que no podemos probar nosotros. Los campos estan en la hoja 3.</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row customHeight="1" ht="78" r="29">
+      <c r="A29" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>BAJA</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>Proveedores de entrega personal</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>¿Confirmas esta lista para dejarla precargada? Entrega local / personal, Uber o delivery, Driver particular, Courier local.</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="E29" s="8" t="inlineStr">
         <is>
           <t>Hoy no hay ninguno cargado, asi que la pantalla de Entrega Personal avisa que faltan configurar. En cualquier caso los podes crear, editar o desactivar vos mismo desde Catalogos → Proveedores.</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F29" s="7" t="inlineStr">
         <is>
           <t/>
         </is>

</xml_diff>